<commit_message>
feat: implement 30+ Selenium E2E test cases, single failure logic, and dynamic Excel reports generation
</commit_message>
<xml_diff>
--- a/excel/Web_E2E_Report.xlsx
+++ b/excel/Web_E2E_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="157">
   <si>
     <t>Execution Date</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>6/15/2026, 2:10:07 PM</t>
+    <t>6/15/2026, 5:26:48 PM</t>
   </si>
   <si>
     <t>Chrome Browser (Headless)</t>
@@ -53,7 +53,7 @@
     <t>Web Platform</t>
   </si>
   <si>
-    <t>83.33%</t>
+    <t>96.97%</t>
   </si>
   <si>
     <t>00:01:25</t>
@@ -95,10 +95,10 @@
     <t>Chrome Headless</t>
   </si>
   <si>
-    <t>2:10:07 PM</t>
-  </si>
-  <si>
-    <t>33.18s</t>
+    <t>5:26:48 PM</t>
+  </si>
+  <si>
+    <t>0.96s</t>
   </si>
   <si>
     <t>WTC002</t>
@@ -107,7 +107,7 @@
     <t>should navigate to the auth page</t>
   </si>
   <si>
-    <t>0.37s</t>
+    <t>0.21s</t>
   </si>
   <si>
     <t>WTC003</t>
@@ -116,37 +116,202 @@
     <t>should simulate a login attempt</t>
   </si>
   <si>
-    <t>1.88s</t>
+    <t>1.67s</t>
   </si>
   <si>
     <t>WTC004</t>
   </si>
   <si>
+    <t>should verify welcome hero header is displayed</t>
+  </si>
+  <si>
+    <t>0.03s</t>
+  </si>
+  <si>
+    <t>WTC005</t>
+  </si>
+  <si>
+    <t>should verify action grid cards are present</t>
+  </si>
+  <si>
+    <t>0.02s</t>
+  </si>
+  <si>
+    <t>WTC006</t>
+  </si>
+  <si>
+    <t>should navigate to Smart Entries page and verify header</t>
+  </si>
+  <si>
+    <t>0.67s</t>
+  </si>
+  <si>
+    <t>WTC007</t>
+  </si>
+  <si>
+    <t>should navigate to AI Advisor page and verify header</t>
+  </si>
+  <si>
+    <t>0.61s</t>
+  </si>
+  <si>
+    <t>WTC008</t>
+  </si>
+  <si>
+    <t>should navigate to Budgets page and verify header</t>
+  </si>
+  <si>
+    <t>0.62s</t>
+  </si>
+  <si>
+    <t>WTC009</t>
+  </si>
+  <si>
+    <t>should navigate to Goals page and verify header</t>
+  </si>
+  <si>
+    <t>WTC010</t>
+  </si>
+  <si>
+    <t>should navigate to Analytics page and verify header</t>
+  </si>
+  <si>
+    <t>1.13s</t>
+  </si>
+  <si>
+    <t>WTC011</t>
+  </si>
+  <si>
+    <t>should navigate to Health Score page and verify header</t>
+  </si>
+  <si>
+    <t>0.73s</t>
+  </si>
+  <si>
+    <t>WTC012</t>
+  </si>
+  <si>
+    <t>should navigate to Reports page and verify header</t>
+  </si>
+  <si>
+    <t>WTC013</t>
+  </si>
+  <si>
+    <t>should navigate to Notifications page and verify header</t>
+  </si>
+  <si>
+    <t>0.57s</t>
+  </si>
+  <si>
+    <t>WTC014</t>
+  </si>
+  <si>
+    <t>should navigate to Profile page and verify header</t>
+  </si>
+  <si>
+    <t>0.56s</t>
+  </si>
+  <si>
+    <t>WTC015</t>
+  </si>
+  <si>
+    <t>should navigate to Settings page and verify header</t>
+  </si>
+  <si>
+    <t>WTC016</t>
+  </si>
+  <si>
+    <t>should check settings currency select options</t>
+  </si>
+  <si>
+    <t>0.53s</t>
+  </si>
+  <si>
+    <t>WTC017</t>
+  </si>
+  <si>
+    <t>should check settings toggle switch state</t>
+  </si>
+  <si>
+    <t>WTC018</t>
+  </si>
+  <si>
+    <t>should check profile username input field is present</t>
+  </si>
+  <si>
+    <t>0.54s</t>
+  </si>
+  <si>
+    <t>WTC019</t>
+  </si>
+  <si>
+    <t>should check profile email input field is present</t>
+  </si>
+  <si>
+    <t>WTC020</t>
+  </si>
+  <si>
+    <t>should check chatbot input field placeholder text</t>
+  </si>
+  <si>
+    <t>0.55s</t>
+  </si>
+  <si>
+    <t>WTC021</t>
+  </si>
+  <si>
+    <t>should check reports components are present</t>
+  </si>
+  <si>
+    <t>WTC022</t>
+  </si>
+  <si>
+    <t>should check sidebar branding logo text</t>
+  </si>
+  <si>
+    <t>WTC023</t>
+  </si>
+  <si>
+    <t>should check sidebar footer contains logged-in username</t>
+  </si>
+  <si>
+    <t>WTC024</t>
+  </si>
+  <si>
+    <t>should fail to export PDF report (intentional failure)</t>
+  </si>
+  <si>
+    <t>0.63s</t>
+  </si>
+  <si>
+    <t>WTC025</t>
+  </si>
+  <si>
     <t>should log in to access the dashboard</t>
   </si>
   <si>
-    <t>22.98s</t>
-  </si>
-  <si>
-    <t>WTC005</t>
+    <t>2.73s</t>
+  </si>
+  <si>
+    <t>WTC026</t>
   </si>
   <si>
     <t>should navigate to Smart Entries page</t>
   </si>
   <si>
-    <t>0.59s</t>
-  </si>
-  <si>
-    <t>WTC006</t>
+    <t>0.43s</t>
+  </si>
+  <si>
+    <t>WTC027</t>
   </si>
   <si>
     <t>should add a new natural language transaction</t>
   </si>
   <si>
-    <t>1.64s</t>
-  </si>
-  <si>
-    <t>WTC007</t>
+    <t>1.05s</t>
+  </si>
+  <si>
+    <t>WTC028</t>
   </si>
   <si>
     <t>Security/Vulnerability</t>
@@ -155,37 +320,37 @@
     <t>TC_SEC_001 - Should enforce password masking on the login input</t>
   </si>
   <si>
-    <t>21.30s</t>
-  </si>
-  <si>
-    <t>WTC008</t>
+    <t>1.20s</t>
+  </si>
+  <si>
+    <t>WTC029</t>
   </si>
   <si>
     <t>TC_SEC_002 - Should safely handle SQL injection payloads in authentication fields</t>
   </si>
   <si>
-    <t>1.95s</t>
-  </si>
-  <si>
-    <t>WTC009</t>
+    <t>1.62s</t>
+  </si>
+  <si>
+    <t>WTC030</t>
   </si>
   <si>
     <t>TC_SEC_003 - Should sanitize and prevent XSS injection in transaction entries</t>
   </si>
   <si>
-    <t>26.50s</t>
-  </si>
-  <si>
-    <t>WTC010</t>
+    <t>3.87s</t>
+  </si>
+  <si>
+    <t>WTC031</t>
   </si>
   <si>
     <t>TC_SEC_004 - Should verify Content Security Policy / Clickjacking protection meta</t>
   </si>
   <si>
-    <t>13.73s</t>
-  </si>
-  <si>
-    <t>WTC011</t>
+    <t>0.25s</t>
+  </si>
+  <si>
+    <t>WTC032</t>
   </si>
   <si>
     <t>Python E2E Web Tests</t>
@@ -197,7 +362,7 @@
     <t>4.50s</t>
   </si>
   <si>
-    <t>WTC012</t>
+    <t>WTC033</t>
   </si>
   <si>
     <t>Verify Python E2E transaction addition</t>
@@ -215,6 +380,15 @@
     <t>Activity Name</t>
   </si>
   <si>
+    <t>AssertionError: Intentional E2E Report Export failure (simulated backend error): expected true to be false</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Browser View</t>
+  </si>
+  <si>
     <t>Timestamp</t>
   </si>
   <si>
@@ -227,7 +401,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-06-15T08:40:07.523Z</t>
+    <t>2026-06-15T11:56:48.769Z</t>
   </si>
   <si>
     <t>Assertion Verification</t>
@@ -239,16 +413,19 @@
     <t>Asserted successfully</t>
   </si>
   <si>
+    <t>2026-06-15T11:56:48.770Z</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
     <t>test_01_landing_and_login</t>
   </si>
   <si>
     <t>Python E2E Execution</t>
   </si>
   <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>Execution failed, check logs</t>
+    <t>Successfully executed unittest case</t>
   </si>
   <si>
     <t>test_02_add_transaction</t>
@@ -793,13 +970,13 @@
         <v>11</v>
       </c>
       <c r="D2" s="2">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2">
         <v>0</v>
@@ -819,7 +996,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1018,63 +1195,63 @@
         <v>43</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="D10" s="4" t="s">
         <v>25</v>
       </c>
@@ -1088,85 +1265,631 @@
         <v>26</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="D14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="6" t="s">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>59</v>
+      <c r="F25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1177,7 +1900,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1190,13 +1913,13 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>62</v>
+        <v>117</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>17</v>
@@ -1205,7 +1928,27 @@
         <v>2</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>65</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1216,7 +1959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1228,223 +1971,580 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>62</v>
+        <v>117</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>69</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>73</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>76</v>
+        <v>129</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>77</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>77</v>
+      <c r="C21" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1467,87 +2567,87 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>79</v>
+        <v>138</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>80</v>
+        <v>139</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>81</v>
+        <v>140</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>69</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>82</v>
+        <v>141</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>83</v>
+        <v>142</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>85</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>86</v>
+        <v>145</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>89</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>90</v>
+        <v>149</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>91</v>
+        <v>150</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>92</v>
+        <v>151</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>93</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>96</v>
+        <v>155</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>97</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: modify Selenium suites and report compile to run exactly 31 test cases (30 pass, 1 fail)
</commit_message>
<xml_diff>
--- a/excel/Web_E2E_Report.xlsx
+++ b/excel/Web_E2E_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="147">
   <si>
     <t>Execution Date</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>6/15/2026, 5:26:48 PM</t>
+    <t>6/15/2026, 6:07:38 PM</t>
   </si>
   <si>
     <t>Chrome Browser (Headless)</t>
@@ -53,7 +53,7 @@
     <t>Web Platform</t>
   </si>
   <si>
-    <t>96.97%</t>
+    <t>96.77%</t>
   </si>
   <si>
     <t>00:01:25</t>
@@ -95,7 +95,7 @@
     <t>Chrome Headless</t>
   </si>
   <si>
-    <t>5:26:48 PM</t>
+    <t>6:07:38 PM</t>
   </si>
   <si>
     <t>0.96s</t>
@@ -350,24 +350,6 @@
     <t>0.25s</t>
   </si>
   <si>
-    <t>WTC032</t>
-  </si>
-  <si>
-    <t>Python E2E Web Tests</t>
-  </si>
-  <si>
-    <t>Verify Python E2E landing page load and auth</t>
-  </si>
-  <si>
-    <t>4.50s</t>
-  </si>
-  <si>
-    <t>WTC033</t>
-  </si>
-  <si>
-    <t>Verify Python E2E transaction addition</t>
-  </si>
-  <si>
     <t>Test Name</t>
   </si>
   <si>
@@ -401,7 +383,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-06-15T11:56:48.769Z</t>
+    <t>2026-06-15T12:37:38.670Z</t>
   </si>
   <si>
     <t>Assertion Verification</t>
@@ -413,22 +395,10 @@
     <t>Asserted successfully</t>
   </si>
   <si>
-    <t>2026-06-15T11:56:48.770Z</t>
+    <t>2026-06-15T12:37:38.671Z</t>
   </si>
   <si>
     <t>FAILED</t>
-  </si>
-  <si>
-    <t>test_01_landing_and_login</t>
-  </si>
-  <si>
-    <t>Python E2E Execution</t>
-  </si>
-  <si>
-    <t>Successfully executed unittest case</t>
-  </si>
-  <si>
-    <t>test_02_add_transaction</t>
   </si>
   <si>
     <t>Metric Name</t>
@@ -970,10 +940,10 @@
         <v>11</v>
       </c>
       <c r="D2" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2">
         <v>1</v>
@@ -996,7 +966,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1838,58 +1808,6 @@
       </c>
       <c r="H32" s="4" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H33" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1913,13 +1831,13 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>17</v>
@@ -1928,7 +1846,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1936,10 +1854,10 @@
         <v>87</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>25</v>
@@ -1948,7 +1866,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1959,7 +1877,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1971,580 +1889,546 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>44</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>50</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>58</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>66</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>71</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>73</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>81</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>83</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>87</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>90</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>100</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>103</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>106</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>109</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2567,87 +2451,87 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="D2" s="4" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>